<commit_message>
5_varying timelags and hyper finished. Save before simulation of 25 hours
</commit_message>
<xml_diff>
--- a/src/case_study/manufacturing/5_best_timelags_and_hyper.xlsx
+++ b/src/case_study/manufacturing/5_best_timelags_and_hyper.xlsx
@@ -425,234 +425,483 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>inputs</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>timelags</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>init_ls</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>opt_ls</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>init_nv</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>opt_nv</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>step</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>init_os</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>init_ls</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>init_nv</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>outputscale</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>lengthscale</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>noise_var</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>mse</t>
+          <t>MSE</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="B2" t="n">
-        <v>40</v>
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2922 Closed Bottom Temperature - Downstream Working End (PV)</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[62.20657   34.67427   56.12179   25.325306   1.269551  72.39474
- 37.030037  96.348854  27.217182   7.0666137 70.665504  17.470806
-  7.0621295 98.645004 ]</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>21.73145884630864</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1043821722269058</v>
+        <v>20.85811614990234</v>
       </c>
       <c r="F2" t="n">
-        <v>4.199195861816406</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>[61.3964    33.702457  55.344246  24.426212   0.6871743 71.57025
- 36.15809   95.52687   26.394566   6.3540993 69.71964   16.571974
-  6.1539016 97.72814  ]</t>
-        </is>
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.03760718926787376</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1704180836677551</v>
+        <v>40</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01230905449545334</v>
+        <v>0.02866045009435398</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B3" t="n">
-        <v>40</v>
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2918 Closed Bottom Temperature - Port 6 (PV)</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[50.58228185 32.88978588 86.20157132 74.03235054  4.3413476  85.50430393
- 58.01983112 62.2998584   0.64384641 40.37423215 60.8368589  21.97767853
- 54.41357935 73.0079821 ]</t>
-        </is>
+        <v>181</v>
+      </c>
+      <c r="D3" t="n">
+        <v>78.28658930787728</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08233899258780107</v>
+        <v>77.39901733398438</v>
       </c>
       <c r="F3" t="n">
-        <v>1.181544423103333</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>[49.72142    31.915602   85.25056    73.244156    3.3244429  84.729126
- 57.232708   61.516968    0.30895278 39.6011     60.07463    21.037651
- 53.637173   72.256165  ]</t>
-        </is>
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.03760718926787376</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1585428267717361</v>
+        <v>40</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01449660149081921</v>
+        <v>0.02866045009435398</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="B4" t="n">
-        <v>40</v>
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2921 Closed Bottom Temperature - Upstream Working End (PV)</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[74.33094537 52.58307723 72.92697402 24.7696846  32.58636627 38.25052765
- 45.45037154  1.49061643  4.04223251 51.14067246 14.92084817 56.66824327
- 53.15050105  7.860884  ]</t>
-        </is>
+        <v>162</v>
+      </c>
+      <c r="D4" t="n">
+        <v>36.47916097783162</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01122095480278519</v>
+        <v>35.49796295166016</v>
       </c>
       <c r="F4" t="n">
-        <v>1.18187415599823</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>[73.443375  51.681618  71.866066  23.899483  31.759188  37.377087
- 44.59343    0.869248   3.1701033 50.3887    14.0058775 55.80463
- 52.315918   7.01218  ]</t>
-        </is>
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.03760718926787376</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02510675042867661</v>
+        <v>40</v>
       </c>
       <c r="I4" t="n">
-        <v>0.01897033819428237</v>
+        <v>0.02866045009435398</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B5" t="n">
-        <v>40</v>
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2923 Filling Pocket Closed Bottom Temperature Centre (PV)</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[63.01012684 35.78032453 56.94965    26.19930949  2.00592453 73.27203661
- 37.87849592 97.18341434 28.04938536  7.93924852 71.42941198 18.34952527
-  7.96527626 99.53659724]</t>
-        </is>
+        <v>49</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5.569804810118381</v>
       </c>
       <c r="E5" t="n">
-        <v>0.04951668728680929</v>
+        <v>4.70089864730835</v>
       </c>
       <c r="F5" t="n">
-        <v>3.364251375198364</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>[62.20657   34.67427   56.12179   25.325306   1.269551  72.39474
- 37.030037  96.348854  27.217182   7.0666137 70.665504  17.470806
-  7.0621295 98.645004 ]</t>
-        </is>
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.03760718926787376</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1043821722269058</v>
+        <v>40</v>
       </c>
       <c r="I5" t="n">
-        <v>0.02028342005791733</v>
+        <v>0.02866045009435398</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10091 Furnace Load</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>122</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.3623340565674829</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.2266871333122253</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H6" t="n">
+        <v>40</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7546 Open Crown Temperature - Port 1 (PV)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>47</v>
+      </c>
+      <c r="D7" t="n">
+        <v>75.92084156845199</v>
+      </c>
+      <c r="E7" t="n">
+        <v>74.99011993408203</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7746 Open Crown Temperature - Port 2 (PV)</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>87</v>
+      </c>
+      <c r="D8" t="n">
+        <v>14.46945482256522</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13.56520748138428</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H8" t="n">
+        <v>40</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="B6" t="n">
-        <v>40</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>[25.68724109 75.14921153 48.79678814 40.30230167 63.99748691 47.41922828
- 83.08421696 64.85549965  3.36815953 35.91233729 89.77890398 11.06595054
- 52.93311747  1.97102943]</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.08606664881780719</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2.540630340576172</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>[24.790354  74.314316  47.945347  39.473675  63.149113  46.527107
- 82.233864  63.961018   2.5122097 35.025154  88.843124  10.136376
- 52.067635   1.4265124]</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>0.1778339743614197</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0.02063503559056429</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>7522 Open Crown Temperature - Port 4 (PV)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>127</v>
+      </c>
+      <c r="D9" t="n">
+        <v>75.97214501656266</v>
+      </c>
+      <c r="E9" t="n">
+        <v>75.13360595703125</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H9" t="n">
+        <v>40</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>7483 Open Crown Temperature - Port 6 (PV)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>43</v>
+      </c>
+      <c r="D10" t="n">
+        <v>84.23122533069872</v>
+      </c>
+      <c r="E10" t="n">
+        <v>83.48426055908203</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H10" t="n">
+        <v>40</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10271 C9 (T012) Upstream Refiner</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>73</v>
+      </c>
+      <c r="D11" t="n">
+        <v>30.03668088682073</v>
+      </c>
+      <c r="E11" t="n">
+        <v>29.2440013885498</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H11" t="n">
+        <v>40</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>7520 Open Crown Temperature - Upstream Working End (PV)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9.759950556053036</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8.933792114257812</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H12" t="n">
+        <v>40</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>9400 Port 2 Gas Flow (SP)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>47</v>
+      </c>
+      <c r="D13" t="n">
+        <v>82.62346114604401</v>
+      </c>
+      <c r="E13" t="n">
+        <v>81.84979248046875</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H13" t="n">
+        <v>40</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>9282 Tweel Position</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" t="n">
+        <v>26.63667666209299</v>
+      </c>
+      <c r="E14" t="n">
+        <v>25.75555992126465</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H14" t="n">
+        <v>40</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.02866045009435398</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>11384 Wobbe Index (Incoming Gas)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>156</v>
+      </c>
+      <c r="D15" t="n">
+        <v>12.32178959646016</v>
+      </c>
+      <c r="E15" t="n">
+        <v>11.66558456420898</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.01743659431867847</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.03760718926787376</v>
+      </c>
+      <c r="H15" t="n">
+        <v>40</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.02866045009435398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final timelags estimated. Now I need to orgabise files
</commit_message>
<xml_diff>
--- a/src/case_study/manufacturing/5_best_timelags_and_hyper.xlsx
+++ b/src/case_study/manufacturing/5_best_timelags_and_hyper.xlsx
@@ -480,25 +480,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>21.73145884630864</v>
+        <v>11.36342811584473</v>
       </c>
       <c r="E2" t="n">
-        <v>20.85811614990234</v>
+        <v>10.37430763244629</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H2" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="3">
@@ -511,25 +511,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D3" t="n">
-        <v>78.28658930787728</v>
+        <v>0.2791543304920197</v>
       </c>
       <c r="E3" t="n">
-        <v>77.39901733398438</v>
+        <v>0.2978042662143707</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H3" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I3" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="4">
@@ -542,25 +542,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>162</v>
+        <v>93</v>
       </c>
       <c r="D4" t="n">
-        <v>36.47916097783162</v>
+        <v>1.992888808250427</v>
       </c>
       <c r="E4" t="n">
-        <v>35.49796295166016</v>
+        <v>1.591455340385437</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H4" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="5">
@@ -573,25 +573,25 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>49</v>
+        <v>189</v>
       </c>
       <c r="D5" t="n">
-        <v>5.569804810118381</v>
+        <v>17.50839614868164</v>
       </c>
       <c r="E5" t="n">
-        <v>4.70089864730835</v>
+        <v>16.54608726501465</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G5" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H5" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I5" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="6">
@@ -604,25 +604,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3623340565674829</v>
+        <v>79.75820922851562</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2266871333122253</v>
+        <v>80.15860748291016</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G6" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H6" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="7">
@@ -635,25 +635,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="D7" t="n">
-        <v>75.92084156845199</v>
+        <v>56.74176406860352</v>
       </c>
       <c r="E7" t="n">
-        <v>74.99011993408203</v>
+        <v>55.77444839477539</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H7" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I7" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="8">
@@ -666,25 +666,25 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="D8" t="n">
-        <v>14.46945482256522</v>
+        <v>53.0740852355957</v>
       </c>
       <c r="E8" t="n">
-        <v>13.56520748138428</v>
+        <v>52.51207733154297</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G8" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H8" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I8" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="9">
@@ -697,25 +697,25 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>127</v>
+        <v>182</v>
       </c>
       <c r="D9" t="n">
-        <v>75.97214501656266</v>
+        <v>94.95172119140625</v>
       </c>
       <c r="E9" t="n">
-        <v>75.13360595703125</v>
+        <v>94.04875183105469</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G9" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H9" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I9" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="10">
@@ -728,25 +728,25 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="D10" t="n">
-        <v>84.23122533069872</v>
+        <v>22.7724723815918</v>
       </c>
       <c r="E10" t="n">
-        <v>83.48426055908203</v>
+        <v>22.41593933105469</v>
       </c>
       <c r="F10" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G10" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H10" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I10" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="11">
@@ -759,25 +759,25 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D11" t="n">
-        <v>30.03668088682073</v>
+        <v>76.47182464599609</v>
       </c>
       <c r="E11" t="n">
-        <v>29.2440013885498</v>
+        <v>75.49275207519531</v>
       </c>
       <c r="F11" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G11" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H11" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I11" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="12">
@@ -790,25 +790,25 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>25</v>
+        <v>119</v>
       </c>
       <c r="D12" t="n">
-        <v>9.759950556053036</v>
+        <v>28.78800964355469</v>
       </c>
       <c r="E12" t="n">
-        <v>8.933792114257812</v>
+        <v>27.89461135864258</v>
       </c>
       <c r="F12" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G12" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H12" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I12" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="13">
@@ -821,25 +821,25 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D13" t="n">
-        <v>82.62346114604401</v>
+        <v>74.50821685791016</v>
       </c>
       <c r="E13" t="n">
-        <v>81.84979248046875</v>
+        <v>73.53043365478516</v>
       </c>
       <c r="F13" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G13" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H13" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I13" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="14">
@@ -852,25 +852,25 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D14" t="n">
-        <v>26.63667666209299</v>
+        <v>24.26650619506836</v>
       </c>
       <c r="E14" t="n">
-        <v>25.75555992126465</v>
+        <v>23.26811981201172</v>
       </c>
       <c r="F14" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G14" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H14" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I14" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
     <row r="15">
@@ -883,25 +883,25 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="D15" t="n">
-        <v>12.32178959646016</v>
+        <v>74.20478820800781</v>
       </c>
       <c r="E15" t="n">
-        <v>11.66558456420898</v>
+        <v>73.26689910888672</v>
       </c>
       <c r="F15" t="n">
-        <v>0.01743659431867847</v>
+        <v>0.04924444109201431</v>
       </c>
       <c r="G15" t="n">
-        <v>0.03760718926787376</v>
+        <v>0.04746058583259583</v>
       </c>
       <c r="H15" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="I15" t="n">
-        <v>0.02866045009435398</v>
+        <v>0.02923732875970147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>